<commit_message>
added wait for loader
</commit_message>
<xml_diff>
--- a/ResourcesBD/ExcelTemplateForOutletCreation.xlsx
+++ b/ResourcesBD/ExcelTemplateForOutletCreation.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="183">
   <si>
     <t>Outlet Code</t>
   </si>
@@ -424,6 +424,150 @@
   </si>
   <si>
     <t>03228174400</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL249EC</t>
+  </si>
+  <si>
+    <t>03539130700</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLA2B6E</t>
+  </si>
+  <si>
+    <t>03540558600</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL7CE9F</t>
+  </si>
+  <si>
+    <t>03541597700</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL59EC1</t>
+  </si>
+  <si>
+    <t>03542875200</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLA9C3D</t>
+  </si>
+  <si>
+    <t>03909766800</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL96B93</t>
+  </si>
+  <si>
+    <t>03911744600</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL4E430</t>
+  </si>
+  <si>
+    <t>03913291900</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLB6B16</t>
+  </si>
+  <si>
+    <t>03915102400</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL3DE0B</t>
+  </si>
+  <si>
+    <t>03662644600</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL5C07A</t>
+  </si>
+  <si>
+    <t>03664407300</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL25C26</t>
+  </si>
+  <si>
+    <t>03666645600</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL4755A</t>
+  </si>
+  <si>
+    <t>03668212900</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLE250D</t>
+  </si>
+  <si>
+    <t>03414844600</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLF8A6D</t>
+  </si>
+  <si>
+    <t>03416154200</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL41797</t>
+  </si>
+  <si>
+    <t>03417353100</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL71CE3</t>
+  </si>
+  <si>
+    <t>03418752100</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLC8E5D</t>
+  </si>
+  <si>
+    <t>03847171700</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLEB58C</t>
+  </si>
+  <si>
+    <t>03847931100</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL7590B</t>
+  </si>
+  <si>
+    <t>03848410000</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLED2A1</t>
+  </si>
+  <si>
+    <t>03848821900</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL23AC9</t>
+  </si>
+  <si>
+    <t>03048873600</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLF7F06</t>
+  </si>
+  <si>
+    <t>03049303400</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL2C4D2</t>
+  </si>
+  <si>
+    <t>03049739000</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLDAA23</t>
+  </si>
+  <si>
+    <t>03050276300</t>
   </si>
 </sst>
 </file>
@@ -1059,7 +1203,7 @@
     </row>
     <row r="2" spans="1:74" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>74</v>
@@ -1086,7 +1230,7 @@
         <v>26.36</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>24.01085412757735</v>
+        <v>24.43591250434271</v>
       </c>
       <c r="S2" s="1" t="s">
         <v>80</v>
@@ -1167,7 +1311,7 @@
         <v>96</v>
       </c>
       <c r="BJ2" s="5" t="s">
-        <v>128</v>
+        <v>176</v>
       </c>
       <c r="BK2" s="1" t="s">
         <v>97</v>
@@ -1181,7 +1325,7 @@
     </row>
     <row r="3" spans="1:74" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
-        <v>129</v>
+        <v>177</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>98</v>
@@ -1208,7 +1352,7 @@
         <v>26.36</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>24.139473632188565</v>
+        <v>24.951090911490727</v>
       </c>
       <c r="S3" s="1" t="s">
         <v>80</v>
@@ -1289,7 +1433,7 @@
         <v>96</v>
       </c>
       <c r="BJ3" s="5" t="s">
-        <v>130</v>
+        <v>178</v>
       </c>
       <c r="BK3" s="1" t="s">
         <v>97</v>
@@ -1303,7 +1447,7 @@
     </row>
     <row r="4" spans="1:74" x14ac:dyDescent="0.35">
       <c r="B4" s="1" t="s">
-        <v>131</v>
+        <v>179</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>99</v>
@@ -1330,7 +1474,7 @@
         <v>26.36</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>24.77904887564629</v>
+        <v>24.55522971073949</v>
       </c>
       <c r="S4" s="1" t="s">
         <v>80</v>
@@ -1411,7 +1555,7 @@
         <v>96</v>
       </c>
       <c r="BJ4" s="5" t="s">
-        <v>132</v>
+        <v>180</v>
       </c>
       <c r="BK4" s="1" t="s">
         <v>97</v>
@@ -1425,7 +1569,7 @@
     </row>
     <row r="5" spans="1:74" x14ac:dyDescent="0.35">
       <c r="B5" s="1" t="s">
-        <v>133</v>
+        <v>181</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>100</v>
@@ -1452,7 +1596,7 @@
         <v>26.36</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>24.23184957564713</v>
+        <v>24.787658661416586</v>
       </c>
       <c r="S5" s="1" t="s">
         <v>80</v>
@@ -1533,7 +1677,7 @@
         <v>96</v>
       </c>
       <c r="BJ5" s="5" t="s">
-        <v>134</v>
+        <v>182</v>
       </c>
       <c r="BK5" s="1" t="s">
         <v>97</v>

</xml_diff>

<commit_message>
Added complete PJP upload flow. Added screen lookup by test ID. Improved Excel download/upload handling. Enhanced UI validation with update confirmation and notification handling. Added support for confirmation dialogs and update result verification.
</commit_message>
<xml_diff>
--- a/ResourcesBD/ExcelTemplateForOutletCreation.xlsx
+++ b/ResourcesBD/ExcelTemplateForOutletCreation.xlsx
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="Excel Template" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913" concurrentManualCount="8"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="122">
   <si>
     <t>Outlet Code</t>
   </si>
@@ -321,709 +321,70 @@
     <t>Hammad Outlet18</t>
   </si>
   <si>
-    <t>Hammad Outlet19</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL65444</t>
-  </si>
-  <si>
-    <t>03409419300</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLC0EFD</t>
-  </si>
-  <si>
-    <t>03410887200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLEA06B</t>
-  </si>
-  <si>
-    <t>03411859600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLABA79</t>
-  </si>
-  <si>
-    <t>03414399000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00001 </t>
-  </si>
-  <si>
     <t>00001</t>
   </si>
   <si>
-    <t>AUTO_OUTLD054F</t>
-  </si>
-  <si>
-    <t>03178270500</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLE2358</t>
-  </si>
-  <si>
-    <t>03179270600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL5FD38</t>
-  </si>
-  <si>
-    <t>03180106700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLC61CF</t>
-  </si>
-  <si>
-    <t>03180933600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL1F7B8</t>
-  </si>
-  <si>
-    <t>03300124100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLCC4FE</t>
-  </si>
-  <si>
-    <t>03301238800</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLF1F08</t>
-  </si>
-  <si>
-    <t>03302260600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLEE7E8</t>
-  </si>
-  <si>
-    <t>03303520000</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL0A15A</t>
-  </si>
-  <si>
-    <t>03223040600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLE0108</t>
-  </si>
-  <si>
-    <t>03225272900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL4B7D4</t>
-  </si>
-  <si>
-    <t>03226759800</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL60D83</t>
-  </si>
-  <si>
-    <t>03228174400</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL249EC</t>
-  </si>
-  <si>
-    <t>03539130700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLA2B6E</t>
-  </si>
-  <si>
-    <t>03540558600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL7CE9F</t>
-  </si>
-  <si>
-    <t>03541597700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL59EC1</t>
-  </si>
-  <si>
-    <t>03542875200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLA9C3D</t>
-  </si>
-  <si>
-    <t>03909766800</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL96B93</t>
-  </si>
-  <si>
-    <t>03911744600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL4E430</t>
-  </si>
-  <si>
-    <t>03913291900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLB6B16</t>
-  </si>
-  <si>
-    <t>03915102400</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL3DE0B</t>
-  </si>
-  <si>
-    <t>03662644600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL5C07A</t>
-  </si>
-  <si>
-    <t>03664407300</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL25C26</t>
-  </si>
-  <si>
-    <t>03666645600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL4755A</t>
-  </si>
-  <si>
-    <t>03668212900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLE250D</t>
-  </si>
-  <si>
-    <t>03414844600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLF8A6D</t>
-  </si>
-  <si>
-    <t>03416154200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL41797</t>
-  </si>
-  <si>
-    <t>03417353100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL71CE3</t>
-  </si>
-  <si>
-    <t>03418752100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLC8E5D</t>
-  </si>
-  <si>
-    <t>03847171700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLEB58C</t>
-  </si>
-  <si>
-    <t>03847931100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL7590B</t>
-  </si>
-  <si>
-    <t>03848410000</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLED2A1</t>
-  </si>
-  <si>
-    <t>03848821900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL23AC9</t>
-  </si>
-  <si>
-    <t>03048873600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLF7F06</t>
-  </si>
-  <si>
-    <t>03049303400</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL2C4D2</t>
-  </si>
-  <si>
-    <t>03049739000</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLDAA23</t>
-  </si>
-  <si>
-    <t>03050276300</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLD07DF</t>
-  </si>
-  <si>
-    <t>03371454000</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLC46D7</t>
-  </si>
-  <si>
-    <t>03372099900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLD57E6</t>
-  </si>
-  <si>
-    <t>03372668100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL91377</t>
-  </si>
-  <si>
-    <t>03373147300</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL53A49</t>
-  </si>
-  <si>
-    <t>03629219700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLDB73D</t>
-  </si>
-  <si>
-    <t>03629839200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLE8F78</t>
-  </si>
-  <si>
-    <t>03630341100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLBC979</t>
-  </si>
-  <si>
-    <t>03630794800</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL33E9F</t>
-  </si>
-  <si>
-    <t>03654907400</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL2D94E</t>
-  </si>
-  <si>
-    <t>03655515200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLF3E41</t>
-  </si>
-  <si>
-    <t>03656015400</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLA9D36</t>
-  </si>
-  <si>
-    <t>03656501400</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLDC589</t>
-  </si>
-  <si>
-    <t>03979754000</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL35075</t>
-  </si>
-  <si>
-    <t>03980335600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL9F4F0</t>
-  </si>
-  <si>
-    <t>03980675900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL3EF47</t>
-  </si>
-  <si>
-    <t>03980977200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLDFB22</t>
-  </si>
-  <si>
-    <t>03885142200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLC0EB8</t>
-  </si>
-  <si>
-    <t>03885925500</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL5364B</t>
-  </si>
-  <si>
-    <t>03886474500</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL75356</t>
-  </si>
-  <si>
-    <t>03887086200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL63E4E</t>
-  </si>
-  <si>
-    <t>03629603500</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLEDECB</t>
-  </si>
-  <si>
-    <t>03630302900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL869D3</t>
-  </si>
-  <si>
-    <t>03630885600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL6CAF4</t>
-  </si>
-  <si>
-    <t>03631406600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL4FDED</t>
-  </si>
-  <si>
-    <t>03083815300</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLC976C</t>
-  </si>
-  <si>
-    <t>03085330100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL863E9</t>
-  </si>
-  <si>
-    <t>03086355000</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLC76EE</t>
-  </si>
-  <si>
-    <t>03087254700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLF9C0F</t>
-  </si>
-  <si>
-    <t>03241908100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL36848</t>
-  </si>
-  <si>
-    <t>03243402000</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL7744F</t>
-  </si>
-  <si>
-    <t>03244487500</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL95D93</t>
-  </si>
-  <si>
-    <t>03245694100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLBE0C6</t>
-  </si>
-  <si>
-    <t>03345728700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL8E3AE</t>
-  </si>
-  <si>
-    <t>03347281700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL92C9B</t>
-  </si>
-  <si>
-    <t>03348403100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL87C9C</t>
-  </si>
-  <si>
-    <t>03349418200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL2D348</t>
-  </si>
-  <si>
-    <t>03780313400</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL60212</t>
-  </si>
-  <si>
-    <t>03781943500</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL05A4E</t>
-  </si>
-  <si>
-    <t>03783731700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLF39A2</t>
-  </si>
-  <si>
-    <t>03785274700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL46C75</t>
-  </si>
-  <si>
-    <t>03363436900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLB1894</t>
-  </si>
-  <si>
-    <t>03364826300</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLE4512</t>
-  </si>
-  <si>
-    <t>03365780200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL26F2F</t>
-  </si>
-  <si>
-    <t>03366778100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL85826</t>
-  </si>
-  <si>
-    <t>03376889500</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLF3EB0</t>
-  </si>
-  <si>
-    <t>03377781100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLE61CD</t>
-  </si>
-  <si>
-    <t>03378544500</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLDB853</t>
-  </si>
-  <si>
-    <t>03379255000</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL88820</t>
-  </si>
-  <si>
-    <t>03128720000</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL5A233</t>
-  </si>
-  <si>
-    <t>03130136900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL3B6C0</t>
-  </si>
-  <si>
-    <t>03131193500</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLAC77B</t>
-  </si>
-  <si>
-    <t>03132451800</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLA1294</t>
-  </si>
-  <si>
-    <t>03466036600</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL007C4</t>
-  </si>
-  <si>
-    <t>03467546900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL33EFE</t>
-  </si>
-  <si>
-    <t>03468681500</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL3CFDC</t>
-  </si>
-  <si>
-    <t>03469679800</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL5A547</t>
-  </si>
-  <si>
-    <t>03490733900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL48F36</t>
-  </si>
-  <si>
-    <t>03491207000</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLD98C7</t>
-  </si>
-  <si>
-    <t>03491615400</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL24664</t>
-  </si>
-  <si>
-    <t>03491958700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLF2236</t>
-  </si>
-  <si>
-    <t>03407763700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL07E57</t>
-  </si>
-  <si>
-    <t>03408819800</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL4C34F</t>
-  </si>
-  <si>
-    <t>03409623100</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLA19EA</t>
-  </si>
-  <si>
-    <t>03410418800</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLE69DF</t>
-  </si>
-  <si>
-    <t>03954672300</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL20346</t>
-  </si>
-  <si>
-    <t>03955191300</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL786EA</t>
-  </si>
-  <si>
-    <t>03955556900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL372CF</t>
-  </si>
-  <si>
-    <t>03955873200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL06003</t>
-  </si>
-  <si>
-    <t>03469757900</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLA858E</t>
-  </si>
-  <si>
-    <t>03470212500</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL5BBC7</t>
-  </si>
-  <si>
-    <t>03470683700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL21F5A</t>
-  </si>
-  <si>
-    <t>03471113700</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL6F3B3</t>
-  </si>
-  <si>
-    <t>03069210000</t>
-  </si>
-  <si>
-    <t>AUTO_OUTLA5556</t>
-  </si>
-  <si>
-    <t>03070041200</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL585BF</t>
-  </si>
-  <si>
-    <t>03070794300</t>
-  </si>
-  <si>
-    <t>AUTO_OUTL13721</t>
-  </si>
-  <si>
-    <t>03071301300</t>
+    <t>AUTO_OUTLA88C8</t>
+  </si>
+  <si>
+    <t>03972648500</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLF324B</t>
+  </si>
+  <si>
+    <t>03973655000</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL4FD95</t>
+  </si>
+  <si>
+    <t>03974281300</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>124</t>
+  </si>
+  <si>
+    <t>125</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL3C102</t>
+  </si>
+  <si>
+    <t>03394468400</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL66E57</t>
+  </si>
+  <si>
+    <t>03395387100</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL9917B</t>
+  </si>
+  <si>
+    <t>03395959800</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL3423B</t>
+  </si>
+  <si>
+    <t>03419093300</t>
+  </si>
+  <si>
+    <t>AUTO_OUTLA7C32</t>
+  </si>
+  <si>
+    <t>03420264500</t>
+  </si>
+  <si>
+    <t>AUTO_OUTL2BAE2</t>
+  </si>
+  <si>
+    <t>03421117000</t>
   </si>
 </sst>
 </file>
@@ -1067,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1075,6 +436,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1355,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BV5"/>
+  <dimension ref="A1:BV4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="10.7265625"/>
@@ -1659,7 +1021,7 @@
     </row>
     <row r="2" spans="1:74" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
-        <v>327</v>
+        <v>116</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>74</v>
@@ -1686,7 +1048,7 @@
         <v>26.36</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>24.878051902407005</v>
+        <v>24.665149954259327</v>
       </c>
       <c r="S2" s="1" t="s">
         <v>80</v>
@@ -1709,6 +1071,9 @@
       <c r="AA2" t="s" s="0">
         <v>84</v>
       </c>
+      <c r="AB2" t="s" s="0">
+        <v>83</v>
+      </c>
       <c r="AC2" t="s" s="0">
         <v>85</v>
       </c>
@@ -1718,6 +1083,9 @@
       <c r="AH2" t="s" s="0">
         <v>84</v>
       </c>
+      <c r="AN2" s="7" t="s">
+        <v>83</v>
+      </c>
       <c r="AP2" s="1" t="s">
         <v>86</v>
       </c>
@@ -1734,7 +1102,7 @@
         <v>90</v>
       </c>
       <c r="AU2" s="5" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="AV2" s="1" t="s">
         <v>91</v>
@@ -1767,10 +1135,16 @@
         <v>96</v>
       </c>
       <c r="BJ2" s="5" t="s">
-        <v>328</v>
+        <v>117</v>
       </c>
       <c r="BK2" s="1" t="s">
         <v>97</v>
+      </c>
+      <c r="BM2" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="BO2" s="1" t="s">
+        <v>107</v>
       </c>
       <c r="BU2" s="1" t="s">
         <v>94</v>
@@ -1781,7 +1155,7 @@
     </row>
     <row r="3" spans="1:74" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
-        <v>329</v>
+        <v>118</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>98</v>
@@ -1808,7 +1182,7 @@
         <v>26.36</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>24.664902173231344</v>
+        <v>24.30760405319391</v>
       </c>
       <c r="S3" s="1" t="s">
         <v>80</v>
@@ -1831,6 +1205,9 @@
       <c r="AA3" t="s" s="0">
         <v>84</v>
       </c>
+      <c r="AB3" t="s" s="0">
+        <v>83</v>
+      </c>
       <c r="AC3" t="s" s="0">
         <v>85</v>
       </c>
@@ -1840,6 +1217,9 @@
       <c r="AH3" t="s" s="0">
         <v>84</v>
       </c>
+      <c r="AN3" s="7" t="s">
+        <v>83</v>
+      </c>
       <c r="AP3" s="1" t="s">
         <v>86</v>
       </c>
@@ -1856,7 +1236,7 @@
         <v>90</v>
       </c>
       <c r="AU3" s="5" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="AV3" s="1" t="s">
         <v>91</v>
@@ -1889,10 +1269,16 @@
         <v>96</v>
       </c>
       <c r="BJ3" s="5" t="s">
-        <v>330</v>
+        <v>119</v>
       </c>
       <c r="BK3" s="1" t="s">
         <v>97</v>
+      </c>
+      <c r="BM3" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="BO3" s="1" t="s">
+        <v>108</v>
       </c>
       <c r="BU3" s="1" t="s">
         <v>94</v>
@@ -1903,7 +1289,7 @@
     </row>
     <row r="4" spans="1:74" x14ac:dyDescent="0.35">
       <c r="B4" s="1" t="s">
-        <v>331</v>
+        <v>120</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>99</v>
@@ -1930,7 +1316,7 @@
         <v>26.36</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>24.980497247428474</v>
+        <v>24.40725232912449</v>
       </c>
       <c r="S4" s="1" t="s">
         <v>80</v>
@@ -1953,6 +1339,9 @@
       <c r="AA4" t="s" s="0">
         <v>84</v>
       </c>
+      <c r="AB4" t="s" s="0">
+        <v>83</v>
+      </c>
       <c r="AC4" t="s" s="0">
         <v>85</v>
       </c>
@@ -1962,6 +1351,9 @@
       <c r="AH4" t="s" s="0">
         <v>84</v>
       </c>
+      <c r="AN4" s="7" t="s">
+        <v>83</v>
+      </c>
       <c r="AP4" s="1" t="s">
         <v>86</v>
       </c>
@@ -1978,7 +1370,7 @@
         <v>90</v>
       </c>
       <c r="AU4" s="5" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="AV4" s="1" t="s">
         <v>91</v>
@@ -2011,137 +1403,21 @@
         <v>96</v>
       </c>
       <c r="BJ4" s="5" t="s">
-        <v>332</v>
+        <v>121</v>
       </c>
       <c r="BK4" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="BM4" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="BO4" s="1" t="s">
+        <v>109</v>
+      </c>
       <c r="BU4" s="1" t="s">
         <v>94</v>
       </c>
       <c r="BV4" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="5" spans="1:74" x14ac:dyDescent="0.35">
-      <c r="B5" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="O5" s="3">
-        <v>26.36</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>24.11215040762057</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="T5" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="U5" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="X5" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Y5" t="s" s="0">
-        <v>83</v>
-      </c>
-      <c r="Z5" t="s" s="0">
-        <v>84</v>
-      </c>
-      <c r="AA5" t="s" s="0">
-        <v>84</v>
-      </c>
-      <c r="AC5" t="s" s="0">
-        <v>85</v>
-      </c>
-      <c r="AD5" t="s" s="0">
-        <v>84</v>
-      </c>
-      <c r="AH5" t="s" s="0">
-        <v>84</v>
-      </c>
-      <c r="AP5" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="AQ5" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="AR5" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="AS5" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="AT5" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="AU5" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="AV5" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="AW5" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="AY5" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="AZ5" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="BA5" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="BC5" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="BD5" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="BE5" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="BF5" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="BG5" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="BJ5" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="BK5" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="BU5" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="BV5" s="1" t="s">
         <v>94</v>
       </c>
     </row>

</xml_diff>